<commit_message>
first code split dump
</commit_message>
<xml_diff>
--- a/data/tuning_plasmid_copy_num/sup_data_2_i_rna.xlsx
+++ b/data/tuning_plasmid_copy_num/sup_data_2_i_rna.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/guillaume/Dropbox (Personal)/Cornell/Publications/Papers/_Rouches-pUC1024/_Resubmission-202203-20220603/SupplementaryTables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User1\IGEM\code\copy-number\data\tuning_plasmid_copy_num\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D6DB8076-B73A-DE43-A1E5-DC46D49192EA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9557E87-964C-4CBF-B634-B0B7A7C02A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12380" yWindow="6400" windowWidth="27240" windowHeight="16440"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="9800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Suplementary Table 3" sheetId="1" r:id="rId1"/>
@@ -22,9 +22,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="372">
   <si>
-    <t>Promoter Sequence (-35 to +1)</t>
-  </si>
-  <si>
     <t>Initial Counts</t>
   </si>
   <si>
@@ -37,9 +34,6 @@
     <t>Copy Number</t>
   </si>
   <si>
-    <t>Predicted Promoter Strength</t>
-  </si>
-  <si>
     <t>TTGCACTGGTGGCCTAACTACGGCTTTACTAGAAGT</t>
   </si>
   <si>
@@ -1136,12 +1130,18 @@
   </si>
   <si>
     <t>TTTCCATGGTGGCCTAACTACGGCTAAGATAGAAGT</t>
+  </si>
+  <si>
+    <t>Predicted Promoter Strength (KbT)</t>
+  </si>
+  <si>
+    <t>Promoter Sequence</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -1975,9 +1975,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F367"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="47" customWidth="1"/>
     <col min="2" max="2" width="19.83203125" customWidth="1"/>
@@ -1987,29 +1987,29 @@
     <col min="6" max="6" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>371</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>6</v>
       </c>
       <c r="B2">
         <v>440</v>
@@ -2027,9 +2027,9 @@
         <v>-2.9499868450952098</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B3">
         <v>996</v>
@@ -2047,9 +2047,9 @@
         <v>-8.4049970400104694</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B4">
         <v>369</v>
@@ -2067,9 +2067,9 @@
         <v>-4.6270446812534001</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B5">
         <v>262</v>
@@ -2087,9 +2087,9 @@
         <v>-4.8118025936827804</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>361</v>
@@ -2107,9 +2107,9 @@
         <v>-3.5826482688240202</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B7">
         <v>591</v>
@@ -2127,9 +2127,9 @@
         <v>-3.9188273111969099</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>220</v>
@@ -2147,9 +2147,9 @@
         <v>-6.4888604298409698</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>323</v>
@@ -2167,9 +2167,9 @@
         <v>-3.9188273111969099</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>1025</v>
@@ -2187,9 +2187,9 @@
         <v>-6.8444581982025499</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B11">
         <v>239</v>
@@ -2207,9 +2207,9 @@
         <v>-6.1574759128918197</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>1131</v>
@@ -2227,9 +2227,9 @@
         <v>-4.5969370710839099</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>934</v>
@@ -2247,9 +2247,9 @@
         <v>-3.34836402023645</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B14">
         <v>9077</v>
@@ -2267,9 +2267,9 @@
         <v>-6.8444581982025499</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B15">
         <v>74</v>
@@ -2287,9 +2287,9 @@
         <v>-6.7580468140217604</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B16">
         <v>2131</v>
@@ -2307,9 +2307,9 @@
         <v>-4.29566016430425</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B17">
         <v>1866</v>
@@ -2327,9 +2327,9 @@
         <v>-4.92832158803306</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B18">
         <v>217</v>
@@ -2347,9 +2347,9 @@
         <v>-3.2512637518748702</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B19">
         <v>267</v>
@@ -2367,9 +2367,9 @@
         <v>-4.3610343281460597</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B20">
         <v>56</v>
@@ -2387,9 +2387,9 @@
         <v>-7.0593237208014301</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B21">
         <v>281</v>
@@ -2407,9 +2407,9 @@
         <v>-8.1037201332308104</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B22">
         <v>467</v>
@@ -2427,9 +2427,9 @@
         <v>-3.0608093450952101</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B23">
         <v>874</v>
@@ -2447,9 +2447,9 @@
         <v>-6.4888604298409698</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B24">
         <v>2293</v>
@@ -2467,9 +2467,9 @@
         <v>-2.7810767603494502</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B25">
         <v>235</v>
@@ -2487,9 +2487,9 @@
         <v>-7.4361565739087698</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B26">
         <v>1802</v>
@@ -2507,9 +2507,9 @@
         <v>-3.34836402023645</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B27">
         <v>11689</v>
@@ -2527,9 +2527,9 @@
         <v>-2.9715311671291098</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B28">
         <v>1841</v>
@@ -2547,9 +2547,9 @@
         <v>-6.6540037914228902</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B29">
         <v>9178</v>
@@ -2567,9 +2567,9 @@
         <v>-2.3039676078070701</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B30">
         <v>74</v>
@@ -2587,9 +2587,9 @@
         <v>-4.8118025936827804</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B31">
         <v>566</v>
@@ -2607,9 +2607,9 @@
         <v>-4.7832243874680902</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B32">
         <v>325</v>
@@ -2627,9 +2627,9 @@
         <v>-5.40543074057544</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B33">
         <v>2395</v>
@@ -2647,9 +2647,9 @@
         <v>-4.2502118281460604</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B34">
         <v>4090</v>
@@ -2667,9 +2667,9 @@
         <v>-3.6496409270161099</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B35">
         <v>1682</v>
@@ -2687,9 +2687,9 @@
         <v>-3.4591865202364498</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B36">
         <v>1265</v>
@@ -2707,9 +2707,9 @@
         <v>-4.5514887349257203</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B37">
         <v>1335</v>
@@ -2727,9 +2727,9 @@
         <v>-4.1267500795584899</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B38">
         <v>405</v>
@@ -2747,9 +2747,9 @@
         <v>-3.6454738366206301</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B39">
         <v>8271</v>
@@ -2767,9 +2767,9 @@
         <v>-3.6496409270161099</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B40">
         <v>11337</v>
@@ -2787,9 +2787,9 @@
         <v>-4.5514887349257203</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B41">
         <v>10116</v>
@@ -2807,9 +2807,9 @@
         <v>-4.5969370710839099</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B42">
         <v>7903</v>
@@ -2827,9 +2827,9 @@
         <v>-3.34836402023645</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B43">
         <v>1895</v>
@@ -2847,9 +2847,9 @@
         <v>-2.0026907010274102</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B44">
         <v>15609</v>
@@ -2867,9 +2867,9 @@
         <v>-5.2645006304059399</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B45">
         <v>871</v>
@@ -2887,9 +2887,9 @@
         <v>-3.4591865202364498</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B46">
         <v>66</v>
@@ -2907,9 +2907,9 @@
         <v>-8.1037201332308104</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B47">
         <v>1965</v>
@@ -2927,9 +2927,9 @@
         <v>-6.8444581982025499</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B48">
         <v>1335</v>
@@ -2947,9 +2947,9 @@
         <v>-2.9715311671291098</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B49">
         <v>66</v>
@@ -2967,9 +2967,9 @@
         <v>-7.1348796671291099</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B50">
         <v>1544</v>
@@ -2987,9 +2987,9 @@
         <v>-4.1267500795584899</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B51">
         <v>385</v>
@@ -3007,9 +3007,9 @@
         <v>-6.6540037914228902</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B52">
         <v>12309</v>
@@ -3027,9 +3027,9 @@
         <v>-4.1267500795584899</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B53">
         <v>2787</v>
@@ -3047,9 +3047,9 @@
         <v>-3.5826482688240202</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B54">
         <v>2601</v>
@@ -3067,9 +3067,9 @@
         <v>-2.9715311671291098</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B55">
         <v>7501</v>
@@ -3087,9 +3087,9 @@
         <v>-3.4591865202364498</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B56">
         <v>108</v>
@@ -3107,9 +3107,9 @@
         <v>-6.4888604298409698</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B57">
         <v>37586</v>
@@ -3127,9 +3127,9 @@
         <v>-3.6496409270161099</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B58">
         <v>275</v>
@@ -3147,9 +3147,9 @@
         <v>-7.0593237208014301</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B59">
         <v>7208</v>
@@ -3167,9 +3167,9 @@
         <v>-4.3172044863381496</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B60">
         <v>968</v>
@@ -3187,9 +3187,9 @@
         <v>-4.92832158803306</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B61">
         <v>1605</v>
@@ -3207,9 +3207,9 @@
         <v>-4.7378671812534003</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B62">
         <v>1240</v>
@@ -3227,9 +3227,9 @@
         <v>-4.5969370710839099</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B63">
         <v>899</v>
@@ -3247,9 +3247,9 @@
         <v>-5.5958851473550997</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B64">
         <v>2316</v>
@@ -3267,9 +3267,9 @@
         <v>-4.3610343281460597</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B65">
         <v>8211</v>
@@ -3287,9 +3287,9 @@
         <v>-4.92832158803306</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B66">
         <v>61</v>
@@ -3307,9 +3307,9 @@
         <v>-6.1875835230613099</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B67">
         <v>1020</v>
@@ -3327,9 +3327,9 @@
         <v>-7.1263163789935202</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B68">
         <v>3579</v>
@@ -3347,9 +3347,9 @@
         <v>-5.2645006304059399</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B69">
         <v>1744</v>
@@ -3367,9 +3367,9 @@
         <v>-5.2645006304059399</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B70">
         <v>296</v>
@@ -3387,9 +3387,9 @@
         <v>-5.8561990061121598</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B71">
         <v>8146</v>
@@ -3407,9 +3407,9 @@
         <v>-7.1263163789935202</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B72">
         <v>1739</v>
@@ -3427,9 +3427,9 @@
         <v>-5.2645006304059399</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B73">
         <v>1052</v>
@@ -3447,9 +3447,9 @@
         <v>-6.1574759128918197</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B74">
         <v>63313</v>
@@ -3467,9 +3467,9 @@
         <v>-4.3172044863381496</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B75">
         <v>1565</v>
@@ -3487,9 +3487,9 @@
         <v>-5.40543074057544</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B76">
         <v>3139</v>
@@ -3507,9 +3507,9 @@
         <v>-5.3753231304059499</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B77">
         <v>14214</v>
@@ -3527,9 +3527,9 @@
         <v>-4.3172044863381496</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B78">
         <v>131</v>
@@ -3547,9 +3547,9 @@
         <v>-6.1574759128918197</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B79">
         <v>553</v>
@@ -3567,9 +3567,9 @@
         <v>-3.72837290441724</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B80">
         <v>54</v>
@@ -3587,9 +3587,9 @@
         <v>-5.0951901784285401</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B81">
         <v>57238</v>
@@ -3607,9 +3607,9 @@
         <v>-3.2728080739087702</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B82">
         <v>909</v>
@@ -3627,9 +3627,9 @@
         <v>-4.92832158803306</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B83">
         <v>6020</v>
@@ -3647,9 +3647,9 @@
         <v>-3.2728080739087702</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B84">
         <v>313005</v>
@@ -3667,9 +3667,9 @@
         <v>-4.6184813931178104</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B85">
         <v>1404</v>
@@ -3687,9 +3687,9 @@
         <v>-2.9715311671291098</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B86">
         <v>4489</v>
@@ -3707,9 +3707,9 @@
         <v>-3.6496409270161099</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B87">
         <v>1135</v>
@@ -3727,9 +3727,9 @@
         <v>-2.3039676078070701</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B88">
         <v>120</v>
@@ -3747,9 +3747,9 @@
         <v>-3.0909169552646998</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B89">
         <v>12772</v>
@@ -3767,9 +3767,9 @@
         <v>-3.2728080739087702</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B90">
         <v>2504</v>
@@ -3787,9 +3787,9 @@
         <v>-4.5514887349257203</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B91">
         <v>1058</v>
@@ -3807,9 +3807,9 @@
         <v>-6.8444581982025499</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B92">
         <v>217</v>
@@ -3827,9 +3827,9 @@
         <v>-6.1875835230613099</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B93">
         <v>146</v>
@@ -3847,9 +3847,9 @@
         <v>-5.78064305978448</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B94">
         <v>13029</v>
@@ -3867,9 +3867,9 @@
         <v>-4.4280269863381498</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B95">
         <v>2095</v>
@@ -3887,9 +3887,9 @@
         <v>-3.8359282434002901</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B96">
         <v>31965</v>
@@ -3907,9 +3907,9 @@
         <v>-4.6184813931178104</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B97">
         <v>1748</v>
@@ -3927,9 +3927,9 @@
         <v>-5.5958851473550997</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B98">
         <v>67450</v>
@@ -3947,9 +3947,9 @@
         <v>-4.6184813931178104</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B99">
         <v>100</v>
@@ -3967,9 +3967,9 @@
         <v>-3.43755106825905</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B100">
         <v>60982</v>
@@ -3987,9 +3987,9 @@
         <v>-4.4280269863381498</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B101">
         <v>1594</v>
@@ -4007,9 +4007,9 @@
         <v>-5.3753231304059499</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B102">
         <v>292</v>
@@ -4027,9 +4027,9 @@
         <v>-5.1146089044172403</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B103">
         <v>242</v>
@@ -4047,9 +4047,9 @@
         <v>-6.6540037914228902</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B104">
         <v>31</v>
@@ -4067,9 +4067,9 @@
         <v>-8.1037201332308104</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B105">
         <v>296</v>
@@ -4087,9 +4087,9 @@
         <v>-5.6872889213663997</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B106">
         <v>76</v>
@@ -4107,9 +4107,9 @@
         <v>-5.2889117462251498</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B107">
         <v>2584</v>
@@ -4127,9 +4127,9 @@
         <v>-3.9188273111969099</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B108">
         <v>7072</v>
@@ -4147,9 +4147,9 @@
         <v>-4.3172044863381496</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B109">
         <v>266</v>
@@ -4167,9 +4167,9 @@
         <v>-8.2145426332307991</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B110">
         <v>1277</v>
@@ -4187,9 +4187,9 @@
         <v>-3.0823536671291101</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B111">
         <v>23</v>
@@ -4207,9 +4207,9 @@
         <v>-4.9527327038522699</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B112">
         <v>2663</v>
@@ -4227,9 +4227,9 @@
         <v>-4.1267500795584899</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B113">
         <v>79</v>
@@ -4247,9 +4247,9 @@
         <v>-5.9670215061121601</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B114">
         <v>1251</v>
@@ -4267,9 +4267,9 @@
         <v>-3.0823536671291101</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B115">
         <v>2004</v>
@@ -4287,9 +4287,9 @@
         <v>-2.11351320102741</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B116">
         <v>2469</v>
@@ -4307,9 +4307,9 @@
         <v>-3.0823536671291101</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B117">
         <v>7010</v>
@@ -4327,9 +4327,9 @@
         <v>-3.2728080739087702</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B118">
         <v>6507</v>
@@ -4347,9 +4347,9 @@
         <v>-4.4280269863381498</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B119">
         <v>105</v>
@@ -4367,9 +4367,9 @@
         <v>-6.63458506543419</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B120">
         <v>11516</v>
@@ -4387,9 +4387,9 @@
         <v>-3.0823536671291101</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B121">
         <v>15167</v>
@@ -4407,9 +4407,9 @@
         <v>-5.3753231304059499</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B122">
         <v>1787</v>
@@ -4427,9 +4427,9 @@
         <v>-7.1263163789935202</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B123">
         <v>171</v>
@@ -4447,9 +4447,9 @@
         <v>-4.7378671812534003</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B124">
         <v>53</v>
@@ -4467,9 +4467,9 @@
         <v>-5.8561990061121598</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B125">
         <v>38</v>
@@ -4487,9 +4487,9 @@
         <v>-5.1146089044172403</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B126">
         <v>48</v>
@@ -4507,9 +4507,9 @@
         <v>-7.4361565739087698</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B127">
         <v>1368</v>
@@ -4527,9 +4527,9 @@
         <v>-4.5514887349257203</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B128">
         <v>481</v>
@@ -4547,9 +4547,9 @@
         <v>-3.2512637518748702</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B129">
         <v>280</v>
@@ -4567,9 +4567,9 @@
         <v>-6.2984060230613101</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B130">
         <v>280</v>
@@ -4587,9 +4587,9 @@
         <v>-6.8250394722138497</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B131">
         <v>51</v>
@@ -4607,9 +4607,9 @@
         <v>-6.9659695823833498</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B132">
         <v>2067</v>
@@ -4627,9 +4627,9 @@
         <v>-2.3039676078070701</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B133">
         <v>1998</v>
@@ -4647,9 +4647,9 @@
         <v>-4.4064826643042503</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B134">
         <v>23</v>
@@ -4667,9 +4667,9 @@
         <v>-6.2984060230613101</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B135">
         <v>245</v>
@@ -4687,9 +4687,9 @@
         <v>-4.7184484552647001</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B136">
         <v>15</v>
@@ -4707,9 +4707,9 @@
         <v>-3.8603393592195001</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B137">
         <v>2058</v>
@@ -4727,9 +4727,9 @@
         <v>-6.8250394722138497</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B138">
         <v>69</v>
@@ -4747,9 +4747,9 @@
         <v>-3.6454738366206301</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B139">
         <v>321</v>
@@ -4767,9 +4767,9 @@
         <v>-5.9670215061121601</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B140">
         <v>7777</v>
@@ -4787,9 +4787,9 @@
         <v>-5.5958851473550997</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B141">
         <v>264</v>
@@ -4807,9 +4807,9 @@
         <v>-2.7810767603494502</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B142">
         <v>470</v>
@@ -4827,9 +4827,9 @@
         <v>-6.63458506543419</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B143">
         <v>51</v>
@@ -4847,9 +4847,9 @@
         <v>-5.1431871106319296</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B144">
         <v>164</v>
@@ -4867,9 +4867,9 @@
         <v>-5.40543074057544</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B145">
         <v>12</v>
@@ -4887,9 +4887,9 @@
         <v>-4.8419102038522697</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B146">
         <v>2239</v>
@@ -4907,9 +4907,9 @@
         <v>-3.2512637518748702</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B147">
         <v>84</v>
@@ -4927,9 +4927,9 @@
         <v>-6.4888604298409698</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B148">
         <v>5</v>
@@ -4947,9 +4947,9 @@
         <v>-5.0951901784285401</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B149">
         <v>908</v>
@@ -4967,9 +4967,9 @@
         <v>-5.5958851473550997</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B150">
         <v>181</v>
@@ -4987,9 +4987,9 @@
         <v>-5.40543074057544</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B151">
         <v>167</v>
@@ -5007,9 +5007,9 @@
         <v>-5.78064305978448</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B152">
         <v>1205</v>
@@ -5027,9 +5027,9 @@
         <v>-6.1120275767336301</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B153">
         <v>6502</v>
@@ -5047,9 +5047,9 @@
         <v>-4.4280269863381498</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B154">
         <v>54</v>
@@ -5067,9 +5067,9 @@
         <v>-6.2984060230613101</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B155">
         <v>301</v>
@@ -5087,9 +5087,9 @@
         <v>-5.1431871106319296</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B156">
         <v>25</v>
@@ -5107,9 +5107,9 @@
         <v>-5.1146089044172403</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B157">
         <v>3091</v>
@@ -5127,9 +5127,9 @@
         <v>-5.0740462236262802</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B158">
         <v>16270</v>
@@ -5147,9 +5147,9 @@
         <v>-5.5657775371856104</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B159">
         <v>1282</v>
@@ -5167,9 +5167,9 @@
         <v>-5.78064305978448</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B160">
         <v>230</v>
@@ -5187,9 +5187,9 @@
         <v>-6.8250394722138497</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B161">
         <v>7</v>
@@ -5207,9 +5207,9 @@
         <v>-5.6657445993325002</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B162">
         <v>36223</v>
@@ -5227,9 +5227,9 @@
         <v>-4.6184813931178104</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B163">
         <v>280</v>
@@ -5247,9 +5247,9 @@
         <v>-3.9188273111969099</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B164">
         <v>74</v>
@@ -5267,9 +5267,9 @@
         <v>-4.6213481869031199</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B165">
         <v>71</v>
@@ -5287,9 +5287,9 @@
         <v>-7.2457021671291102</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B166">
         <v>56</v>
@@ -5307,9 +5307,9 @@
         <v>-4.1052057575245904</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B167">
         <v>143</v>
@@ -5327,9 +5327,9 @@
         <v>-6.1120275767336301</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B168">
         <v>62</v>
@@ -5347,9 +5347,9 @@
         <v>-5.1146089044172403</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B169">
         <v>523</v>
@@ -5367,9 +5367,9 @@
         <v>-5.4987848789935203</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B170">
         <v>6158</v>
@@ -5387,9 +5387,9 @@
         <v>-4.83334691571668</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B171">
         <v>317</v>
@@ -5407,9 +5407,9 @@
         <v>-5.8107506699539702</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B172">
         <v>158</v>
@@ -5427,9 +5427,9 @@
         <v>-6.1120275767336301</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B173">
         <v>229</v>
@@ -5447,9 +5447,9 @@
         <v>-6.54318129142289</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B174">
         <v>641</v>
@@ -5467,9 +5467,9 @@
         <v>-4.5299444128918198</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B175">
         <v>1853</v>
@@ -5487,9 +5487,9 @@
         <v>-5.6872889213663997</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B176">
         <v>17</v>
@@ -5507,9 +5507,9 @@
         <v>-3.2470966614793899</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B177">
         <v>468</v>
@@ -5527,9 +5527,9 @@
         <v>-6.8250394722138497</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B178">
         <v>757</v>
@@ -5547,9 +5547,9 @@
         <v>-4.83334691571668</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B179">
         <v>25</v>
@@ -5567,9 +5567,9 @@
         <v>-3.56322954283532</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B180">
         <v>61</v>
@@ -5587,9 +5587,9 @@
         <v>-5.9971291162816502</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B181">
         <v>12</v>
@@ -5607,9 +5607,9 @@
         <v>-5.0951901784285401</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B182">
         <v>213</v>
@@ -5627,9 +5627,9 @@
         <v>-6.54318129142289</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B183">
         <v>43</v>
@@ -5647,9 +5647,9 @@
         <v>-4.3416156021573604</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B184">
         <v>2073</v>
@@ -5667,9 +5667,9 @@
         <v>-5.87561773210086</v>
       </c>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B185">
         <v>7952</v>
@@ -5687,9 +5687,9 @@
         <v>-5.5657775371856104</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B186">
         <v>85</v>
@@ -5707,9 +5707,9 @@
         <v>-6.8688693140217598</v>
       </c>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B187">
         <v>497</v>
@@ -5727,9 +5727,9 @@
         <v>-7.4577008959426703</v>
       </c>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B188">
         <v>35</v>
@@ -5747,9 +5747,9 @@
         <v>-6.2984060230613101</v>
       </c>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B189">
         <v>712</v>
@@ -5767,9 +5767,9 @@
         <v>-4.83334691571668</v>
       </c>
     </row>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B190">
         <v>75321</v>
@@ -5787,9 +5787,9 @@
         <v>-5.5657775371856104</v>
       </c>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B191">
         <v>12</v>
@@ -5807,9 +5807,9 @@
         <v>-5.6657445993325002</v>
       </c>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B192">
         <v>35</v>
@@ -5827,9 +5827,9 @@
         <v>-5.1431871106319296</v>
       </c>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B193">
         <v>2181</v>
@@ -5847,9 +5847,9 @@
         <v>-6.9358619722138499</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B194">
         <v>1870</v>
@@ -5867,9 +5867,9 @@
         <v>-6.54318129142289</v>
       </c>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B195">
         <v>238</v>
@@ -5887,9 +5887,9 @@
         <v>-6.9659695823833498</v>
       </c>
     </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B196">
         <v>4137</v>
@@ -5907,9 +5907,9 @@
         <v>-7.4577008959426703</v>
       </c>
     </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B197">
         <v>89</v>
@@ -5927,9 +5927,9 @@
         <v>-5.3838864185415396</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B198">
         <v>456</v>
@@ -5947,9 +5947,9 @@
         <v>-5.6872889213663997</v>
       </c>
     </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B199">
         <v>3</v>
@@ -5967,9 +5967,9 @@
         <v>-5.4050303733438003</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B200">
         <v>252</v>
@@ -5987,9 +5987,9 @@
         <v>-5.4987848789935203</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B201">
         <v>33</v>
@@ -6007,9 +6007,9 @@
         <v>-5.1431871106319296</v>
       </c>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B202">
         <v>534</v>
@@ -6027,9 +6027,9 @@
         <v>-7.4577008959426703</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B203">
         <v>930</v>
@@ -6047,9 +6047,9 @@
         <v>-7.1263163789935202</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B204">
         <v>46</v>
@@ -6067,9 +6067,9 @@
         <v>-5.4793661530048201</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B205">
         <v>975</v>
@@ -6087,9 +6087,9 @@
         <v>-3.8645064496149799</v>
       </c>
     </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B206">
         <v>41</v>
@@ -6107,9 +6107,9 @@
         <v>-6.3527268846432303</v>
       </c>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B207">
         <v>426</v>
@@ -6127,9 +6127,9 @@
         <v>-5.6851633253212004</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B208">
         <v>13</v>
@@ -6147,9 +6147,9 @@
         <v>-6.0424863224963401</v>
       </c>
     </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B209">
         <v>372</v>
@@ -6167,9 +6167,9 @@
         <v>-6.3527268846432303</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B210">
         <v>4</v>
@@ -6187,9 +6187,9 @@
         <v>-5.2060126784285403</v>
       </c>
     </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B211">
         <v>69</v>
@@ -6207,9 +6207,9 @@
         <v>-6.63458506543419</v>
       </c>
     </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B212">
         <v>284</v>
@@ -6227,9 +6227,9 @@
         <v>-5.78064305978448</v>
       </c>
     </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B213">
         <v>284</v>
@@ -6247,9 +6247,9 @@
         <v>-6.9358619722138499</v>
       </c>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B214">
         <v>451</v>
@@ -6267,9 +6267,9 @@
         <v>-5.87561773210086</v>
       </c>
     </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B215">
         <v>110</v>
@@ -6287,9 +6287,9 @@
         <v>-7.1564239891630104</v>
       </c>
     </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B216">
         <v>381</v>
@@ -6307,9 +6307,9 @@
         <v>-6.54318129142289</v>
       </c>
     </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B217">
         <v>111</v>
@@ -6327,9 +6327,9 @@
         <v>-3.8645064496149799</v>
       </c>
     </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B218">
         <v>10</v>
@@ -6347,9 +6347,9 @@
         <v>-5.2060126784285403</v>
       </c>
     </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B219">
         <v>267</v>
@@ -6367,9 +6367,9 @@
         <v>-6.1120275767336301</v>
       </c>
     </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B220">
         <v>53</v>
@@ -6387,9 +6387,9 @@
         <v>-5.3964670852082</v>
       </c>
     </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B221">
         <v>4301</v>
@@ -6407,9 +6407,9 @@
         <v>-5.2101797688240197</v>
       </c>
     </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B222">
         <v>3</v>
@@ -6427,9 +6427,9 @@
         <v>-6.1834164326658296</v>
       </c>
     </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B223">
         <v>372</v>
@@ -6447,9 +6447,9 @@
         <v>-5.4793661530048201</v>
       </c>
     </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B224">
         <v>90</v>
@@ -6467,9 +6467,9 @@
         <v>-4.9527327038522699</v>
       </c>
     </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B225">
         <v>223</v>
@@ -6487,9 +6487,9 @@
         <v>-5.87561773210086</v>
       </c>
     </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B226">
         <v>43</v>
@@ -6507,9 +6507,9 @@
         <v>-5.6851633253212004</v>
       </c>
     </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B227">
         <v>1722</v>
@@ -6527,9 +6527,9 @@
         <v>-4.5320700089370201</v>
       </c>
     </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B228">
         <v>488</v>
@@ -6547,9 +6547,9 @@
         <v>-6.9358619722138499</v>
       </c>
     </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B229">
         <v>18</v>
@@ -6567,9 +6567,9 @@
         <v>-4.32007128012346</v>
       </c>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B230">
         <v>124</v>
@@ -6587,9 +6587,9 @@
         <v>-3.8645064496149799</v>
       </c>
     </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B231">
         <v>82</v>
@@ -6607,9 +6607,9 @@
         <v>-5.8107506699539702</v>
       </c>
     </row>
-    <row r="232" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B232">
         <v>494</v>
@@ -6627,9 +6627,9 @@
         <v>-5.2101797688240197</v>
       </c>
     </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B233">
         <v>80</v>
@@ -6647,9 +6647,9 @@
         <v>-4.3416156021573604</v>
       </c>
     </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B234">
         <v>206</v>
@@ -6667,9 +6667,9 @@
         <v>-4.5320700089370201</v>
       </c>
     </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B235">
         <v>25</v>
@@ -6687,9 +6687,9 @@
         <v>-5.8107506699539702</v>
       </c>
     </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B236">
         <v>193</v>
@@ -6707,9 +6707,9 @@
         <v>-4.5320700089370201</v>
       </c>
     </row>
-    <row r="237" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B237">
         <v>1485</v>
@@ -6727,9 +6727,9 @@
         <v>-4.83334691571668</v>
       </c>
     </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B238">
         <v>160</v>
@@ -6747,9 +6747,9 @@
         <v>-5.01972536204436</v>
       </c>
     </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B239">
         <v>1139</v>
@@ -6767,9 +6767,9 @@
         <v>-7.1564239891630104</v>
       </c>
     </row>
-    <row r="240" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B240">
         <v>51</v>
@@ -6787,9 +6787,9 @@
         <v>-5.5901886530048097</v>
       </c>
     </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B241">
         <v>48</v>
@@ -6807,9 +6807,9 @@
         <v>-4.9241544976375797</v>
       </c>
     </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B242">
         <v>245</v>
@@ -6827,9 +6827,9 @@
         <v>-5.87561773210086</v>
       </c>
     </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B243">
         <v>95</v>
@@ -6847,9 +6847,9 @@
         <v>-5.6851633253212004</v>
       </c>
     </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B244">
         <v>945</v>
@@ -6867,9 +6867,9 @@
         <v>-7.4577008959426703</v>
       </c>
     </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B245">
         <v>32960</v>
@@ -6887,9 +6887,9 @@
         <v>-6.1790202349257202</v>
       </c>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B246">
         <v>2</v>
@@ -6907,9 +6907,9 @@
         <v>-4.32007128012346</v>
       </c>
     </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B247">
         <v>90</v>
@@ -6927,9 +6927,9 @@
         <v>-4.8419102038522697</v>
       </c>
     </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B248">
         <v>84</v>
@@ -6947,9 +6947,9 @@
         <v>-3.0608093450952101</v>
       </c>
     </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B249">
         <v>98</v>
@@ -6967,9 +6967,9 @@
         <v>-5.5901886530048097</v>
       </c>
     </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B250">
         <v>234</v>
@@ -6987,9 +6987,9 @@
         <v>-3.8645064496149799</v>
       </c>
     </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B251">
         <v>15</v>
@@ -7007,9 +7007,9 @@
         <v>-5.8714506417053798</v>
       </c>
     </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B252">
         <v>833</v>
@@ -7027,9 +7027,9 @@
         <v>-3.4591865202364498</v>
       </c>
     </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B253">
         <v>58</v>
@@ -7047,9 +7047,9 @@
         <v>-5.5901886530048097</v>
       </c>
     </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B254">
         <v>7</v>
@@ -7067,9 +7067,9 @@
         <v>-6.4846933394454904</v>
       </c>
     </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B255">
         <v>150</v>
@@ -7087,9 +7087,9 @@
         <v>-7.1564239891630104</v>
       </c>
     </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B256">
         <v>92</v>
@@ -7107,9 +7107,9 @@
         <v>-6.3527268846432303</v>
       </c>
     </row>
-    <row r="257" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B257">
         <v>66</v>
@@ -7127,9 +7127,9 @@
         <v>-6.0619050484850403</v>
       </c>
     </row>
-    <row r="258" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B258">
         <v>280</v>
@@ -7147,9 +7147,9 @@
         <v>-3.56322954283532</v>
       </c>
     </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B259">
         <v>11</v>
@@ -7167,9 +7167,9 @@
         <v>-6.8688693140217598</v>
       </c>
     </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B260">
         <v>4119</v>
@@ -7187,9 +7187,9 @@
         <v>-6.1790202349257202</v>
       </c>
     </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B261">
         <v>495</v>
@@ -7207,9 +7207,9 @@
         <v>-4.5320700089370201</v>
       </c>
     </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B262">
         <v>36</v>
@@ -7227,9 +7227,9 @@
         <v>-5.8107506699539702</v>
       </c>
     </row>
-    <row r="263" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B263">
         <v>23</v>
@@ -7247,9 +7247,9 @@
         <v>-5.4793661530048201</v>
       </c>
     </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B264">
         <v>396</v>
@@ -7267,9 +7267,9 @@
         <v>-5.5901886530048097</v>
       </c>
     </row>
-    <row r="265" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B265">
         <v>10</v>
@@ -7287,9 +7287,9 @@
         <v>-4.65145579707261</v>
       </c>
     </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B266">
         <v>15</v>
@@ -7307,9 +7307,9 @@
         <v>-4.9980899100669598</v>
       </c>
     </row>
-    <row r="267" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B267">
         <v>1661</v>
@@ -7327,9 +7327,9 @@
         <v>-5.3753231304059499</v>
       </c>
     </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B268">
         <v>241</v>
@@ -7347,9 +7347,9 @@
         <v>-7.1564239891630104</v>
       </c>
     </row>
-    <row r="269" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B269">
         <v>69</v>
@@ -7367,9 +7367,9 @@
         <v>-5.4793661530048201</v>
       </c>
     </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B270">
         <v>924</v>
@@ -7387,9 +7387,9 @@
         <v>-5.2101797688240197</v>
       </c>
     </row>
-    <row r="271" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B271">
         <v>43</v>
@@ -7407,9 +7407,9 @@
         <v>-5.6851633253212004</v>
       </c>
     </row>
-    <row r="272" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B272">
         <v>61</v>
@@ -7427,9 +7427,9 @@
         <v>-5.8561990061121598</v>
       </c>
     </row>
-    <row r="273" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B273">
         <v>1</v>
@@ -7447,9 +7447,9 @@
         <v>-5.8520319157166796</v>
       </c>
     </row>
-    <row r="274" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B274">
         <v>530</v>
@@ -7467,9 +7467,9 @@
         <v>-4.0296498111969097</v>
       </c>
     </row>
-    <row r="275" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B275">
         <v>35</v>
@@ -7487,9 +7487,9 @@
         <v>-4.7832243874680902</v>
       </c>
     </row>
-    <row r="276" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B276">
         <v>1677</v>
@@ -7507,9 +7507,9 @@
         <v>-5.7067076473550999</v>
       </c>
     </row>
-    <row r="277" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B277">
         <v>3731</v>
@@ -7527,9 +7527,9 @@
         <v>-6.1790202349257202</v>
       </c>
     </row>
-    <row r="278" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B278">
         <v>238</v>
@@ -7547,9 +7547,9 @@
         <v>-4.9089028620443598</v>
       </c>
     </row>
-    <row r="279" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B279">
         <v>22</v>
@@ -7567,9 +7567,9 @@
         <v>-4.4276266191065101</v>
       </c>
     </row>
-    <row r="280" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B280">
         <v>56</v>
@@ -7587,9 +7587,9 @@
         <v>-3.6740520428353198</v>
       </c>
     </row>
-    <row r="281" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B281">
         <v>44</v>
@@ -7607,9 +7607,9 @@
         <v>-5.9670215061121601</v>
       </c>
     </row>
-    <row r="282" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B282">
         <v>497</v>
@@ -7627,9 +7627,9 @@
         <v>-5.2101797688240197</v>
       </c>
     </row>
-    <row r="283" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B283">
         <v>46</v>
@@ -7647,9 +7647,9 @@
         <v>-3.0608093450952101</v>
       </c>
     </row>
-    <row r="284" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B284">
         <v>72</v>
@@ -7667,9 +7667,9 @@
         <v>-5.2060126784285403</v>
       </c>
     </row>
-    <row r="285" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B285">
         <v>262</v>
@@ -7687,9 +7687,9 @@
         <v>-6.9358619722138499</v>
       </c>
     </row>
-    <row r="286" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B286">
         <v>28</v>
@@ -7707,9 +7707,9 @@
         <v>-5.3964670852082</v>
       </c>
     </row>
-    <row r="287" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B287">
         <v>20</v>
@@ -7727,9 +7727,9 @@
         <v>-3.56322954283532</v>
       </c>
     </row>
-    <row r="288" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B288">
         <v>4</v>
@@ -7747,9 +7747,9 @@
         <v>-4.0507937659991704</v>
       </c>
     </row>
-    <row r="289" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B289">
         <v>112</v>
@@ -7767,9 +7767,9 @@
         <v>-4.9089028620443598</v>
       </c>
     </row>
-    <row r="290" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B290">
         <v>476</v>
@@ -7787,9 +7787,9 @@
         <v>-5.30833047221385</v>
       </c>
     </row>
-    <row r="291" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B291">
         <v>315</v>
@@ -7807,9 +7807,9 @@
         <v>-5.9215731699539704</v>
       </c>
     </row>
-    <row r="292" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B292">
         <v>66</v>
@@ -7827,9 +7827,9 @@
         <v>-5.9215731699539704</v>
       </c>
     </row>
-    <row r="293" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B293">
         <v>7731</v>
@@ -7847,9 +7847,9 @@
         <v>-6.1790202349257202</v>
       </c>
     </row>
-    <row r="294" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B294">
         <v>1066</v>
@@ -7867,9 +7867,9 @@
         <v>-4.9089028620443598</v>
       </c>
     </row>
-    <row r="295" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B295">
         <v>28</v>
@@ -7887,9 +7887,9 @@
         <v>-3.6740520428353198</v>
       </c>
     </row>
-    <row r="296" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B296">
         <v>12</v>
@@ -7907,9 +7907,9 @@
         <v>-5.2060126784285403</v>
       </c>
     </row>
-    <row r="297" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B297">
         <v>23</v>
@@ -7927,9 +7927,9 @@
         <v>-6.6751477462251501</v>
       </c>
     </row>
-    <row r="298" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B298">
         <v>6</v>
@@ -7947,9 +7947,9 @@
         <v>-4.2371722123268496</v>
       </c>
     </row>
-    <row r="299" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B299">
         <v>865</v>
@@ -7967,9 +7967,9 @@
         <v>-5.8777433281460603</v>
       </c>
     </row>
-    <row r="300" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B300">
         <v>58</v>
@@ -7987,9 +7987,9 @@
         <v>-6.343763229276</v>
       </c>
     </row>
-    <row r="301" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B301">
         <v>30</v>
@@ -8007,9 +8007,9 @@
         <v>-5.9215731699539704</v>
       </c>
     </row>
-    <row r="302" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B302">
         <v>4</v>
@@ -8027,9 +8027,9 @@
         <v>-6.6751477462251501</v>
       </c>
     </row>
-    <row r="303" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="B303">
         <v>1048</v>
@@ -8047,9 +8047,9 @@
         <v>-5.8777433281460603</v>
       </c>
     </row>
-    <row r="304" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B304">
         <v>427</v>
@@ -8067,9 +8067,9 @@
         <v>-5.5743408253212001</v>
       </c>
     </row>
-    <row r="305" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="B305">
         <v>8676</v>
@@ -8087,9 +8087,9 @@
         <v>-5.8777433281460603</v>
       </c>
     </row>
-    <row r="306" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B306">
         <v>1693</v>
@@ -8107,9 +8107,9 @@
         <v>-4.6428925089370203</v>
       </c>
     </row>
-    <row r="307" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B307">
         <v>145</v>
@@ -8127,9 +8127,9 @@
         <v>-4.9089028620443598</v>
       </c>
     </row>
-    <row r="308" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B308">
         <v>1373</v>
@@ -8147,9 +8147,9 @@
         <v>-4.2201042179765702</v>
       </c>
     </row>
-    <row r="309" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="B309">
         <v>276</v>
@@ -8167,9 +8167,9 @@
         <v>-4.0296498111969097</v>
       </c>
     </row>
-    <row r="310" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B310">
         <v>66</v>
@@ -8187,9 +8187,9 @@
         <v>-5.6202962631743096</v>
       </c>
     </row>
-    <row r="311" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B311">
         <v>66</v>
@@ -8207,9 +8207,9 @@
         <v>-5.9215731699539704</v>
       </c>
     </row>
-    <row r="312" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B312">
         <v>6</v>
@@ -8227,9 +8227,9 @@
         <v>-5.6202962631743096</v>
       </c>
     </row>
-    <row r="313" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B313">
         <v>280</v>
@@ -8247,9 +8247,9 @@
         <v>-4.6428925089370203</v>
       </c>
     </row>
-    <row r="314" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B314">
         <v>33</v>
@@ -8267,9 +8267,9 @@
         <v>-4.0507937659991704</v>
       </c>
     </row>
-    <row r="315" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="315" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B315">
         <v>67</v>
@@ -8287,9 +8287,9 @@
         <v>-3.56322954283532</v>
       </c>
     </row>
-    <row r="316" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="316" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B316">
         <v>155</v>
@@ -8307,9 +8307,9 @@
         <v>-7.2672464891630097</v>
       </c>
     </row>
-    <row r="317" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="B317">
         <v>120</v>
@@ -8327,9 +8327,9 @@
         <v>-7.2672464891630097</v>
       </c>
     </row>
-    <row r="318" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="318" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B318">
         <v>1114</v>
@@ -8347,9 +8347,9 @@
         <v>-7.2672464891630097</v>
       </c>
     </row>
-    <row r="319" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="319" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B319">
         <v>58</v>
@@ -8367,9 +8367,9 @@
         <v>-5.30833047221385</v>
       </c>
     </row>
-    <row r="320" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="320" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B320">
         <v>5</v>
@@ -8387,9 +8387,9 @@
         <v>-5.2889117462251498</v>
       </c>
     </row>
-    <row r="321" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="B321">
         <v>30</v>
@@ -8407,9 +8407,9 @@
         <v>-3.6740520428353198</v>
       </c>
     </row>
-    <row r="322" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="322" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A322" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B322">
         <v>3</v>
@@ -8427,9 +8427,9 @@
         <v>-6.6751477462251501</v>
       </c>
     </row>
-    <row r="323" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="323" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A323" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B323">
         <v>202</v>
@@ -8447,9 +8447,9 @@
         <v>-4.6428925089370203</v>
       </c>
     </row>
-    <row r="324" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="324" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A324" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="B324">
         <v>2001</v>
@@ -8467,9 +8467,9 @@
         <v>-5.8777433281460603</v>
       </c>
     </row>
-    <row r="325" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="325" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A325" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B325">
         <v>285</v>
@@ -8487,9 +8487,9 @@
         <v>-3.6740520428353198</v>
       </c>
     </row>
-    <row r="326" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="326" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A326" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B326">
         <v>1565</v>
@@ -8507,9 +8507,9 @@
         <v>-4.2201042179765702</v>
       </c>
     </row>
-    <row r="327" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A327" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B327">
         <v>12532</v>
@@ -8527,9 +8527,9 @@
         <v>-4.2201042179765702</v>
       </c>
     </row>
-    <row r="328" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="328" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B328">
         <v>49</v>
@@ -8547,9 +8547,9 @@
         <v>-5.5743408253212001</v>
       </c>
     </row>
-    <row r="329" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="329" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A329" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B329">
         <v>376</v>
@@ -8567,9 +8567,9 @@
         <v>-4.3416156021573604</v>
       </c>
     </row>
-    <row r="330" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="330" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A330" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B330">
         <v>46</v>
@@ -8587,9 +8587,9 @@
         <v>-6.63458506543419</v>
       </c>
     </row>
-    <row r="331" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="331" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A331" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B331">
         <v>2562</v>
@@ -8607,9 +8607,9 @@
         <v>-4.0296498111969097</v>
       </c>
     </row>
-    <row r="332" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="332" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A332" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B332">
         <v>272</v>
@@ -8627,9 +8627,9 @@
         <v>-4.0296498111969097</v>
       </c>
     </row>
-    <row r="333" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="333" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A333" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B333">
         <v>485</v>
@@ -8647,9 +8647,9 @@
         <v>-4.6428925089370203</v>
       </c>
     </row>
-    <row r="334" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="334" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A334" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B334">
         <v>313</v>
@@ -8667,9 +8667,9 @@
         <v>-5.4987848789935203</v>
       </c>
     </row>
-    <row r="335" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="335" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A335" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B335">
         <v>247</v>
@@ -8687,9 +8687,9 @@
         <v>-7.2672464891630097</v>
       </c>
     </row>
-    <row r="336" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A336" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B336">
         <v>870</v>
@@ -8707,9 +8707,9 @@
         <v>-5.7067076473550999</v>
       </c>
     </row>
-    <row r="337" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A337" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="B337">
         <v>4290</v>
@@ -8727,9 +8727,9 @@
         <v>-5.8971620541347596</v>
       </c>
     </row>
-    <row r="338" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A338" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B338">
         <v>4724</v>
@@ -8747,9 +8747,9 @@
         <v>-5.8971620541347596</v>
       </c>
     </row>
-    <row r="339" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="339" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A339" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B339">
         <v>2511</v>
@@ -8767,9 +8767,9 @@
         <v>-5.4987848789935203</v>
       </c>
     </row>
-    <row r="340" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="340" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A340" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B340">
         <v>878</v>
@@ -8787,9 +8787,9 @@
         <v>-5.7067076473550999</v>
       </c>
     </row>
-    <row r="341" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A341" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B341">
         <v>2775</v>
@@ -8807,9 +8807,9 @@
         <v>-4.2201042179765702</v>
       </c>
     </row>
-    <row r="342" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A342" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B342">
         <v>6</v>
@@ -8827,9 +8827,9 @@
         <v>-4.9527327038522699</v>
       </c>
     </row>
-    <row r="343" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A343" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B343">
         <v>259</v>
@@ -8847,9 +8847,9 @@
         <v>-3.2512637518748702</v>
       </c>
     </row>
-    <row r="344" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="344" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A344" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B344">
         <v>8600</v>
@@ -8867,9 +8867,9 @@
         <v>-5.8971620541347596</v>
       </c>
     </row>
-    <row r="345" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="345" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A345" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B345">
         <v>39768</v>
@@ -8887,9 +8887,9 @@
         <v>-5.8971620541347596</v>
       </c>
     </row>
-    <row r="346" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A346" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="B346">
         <v>267</v>
@@ -8907,9 +8907,9 @@
         <v>-5.01972536204436</v>
       </c>
     </row>
-    <row r="347" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="347" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A347" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B347">
         <v>17</v>
@@ -8927,9 +8927,9 @@
         <v>-6.9659695823833498</v>
       </c>
     </row>
-    <row r="348" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="348" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A348" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B348">
         <v>7796</v>
@@ -8947,9 +8947,9 @@
         <v>-5.7067076473550999</v>
       </c>
     </row>
-    <row r="349" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="349" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A349" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B349">
         <v>4</v>
@@ -8967,9 +8967,9 @@
         <v>-5.8520319157166796</v>
       </c>
     </row>
-    <row r="350" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A350" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B350">
         <v>30</v>
@@ -8987,9 +8987,9 @@
         <v>-4.3416156021573604</v>
       </c>
     </row>
-    <row r="351" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="351" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A351" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B351">
         <v>115</v>
@@ -9007,9 +9007,9 @@
         <v>-5.01972536204436</v>
       </c>
     </row>
-    <row r="352" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="352" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A352" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B352">
         <v>2</v>
@@ -9027,9 +9027,9 @@
         <v>-5.3294744270161098</v>
       </c>
     </row>
-    <row r="353" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="353" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A353" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B353">
         <v>9222</v>
@@ -9047,9 +9047,9 @@
         <v>-5.9885658281460596</v>
       </c>
     </row>
-    <row r="354" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="354" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A354" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B354">
         <v>1062</v>
@@ -9067,9 +9067,9 @@
         <v>-5.01972536204436</v>
       </c>
     </row>
-    <row r="355" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="355" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A355" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B355">
         <v>217</v>
@@ -9087,9 +9087,9 @@
         <v>-5.6872889213663997</v>
       </c>
     </row>
-    <row r="356" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="356" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A356" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B356">
         <v>1022</v>
@@ -9107,9 +9107,9 @@
         <v>-5.9885658281460596</v>
       </c>
     </row>
-    <row r="357" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="357" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A357" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B357">
         <v>213</v>
@@ -9127,9 +9127,9 @@
         <v>-5.3964670852082</v>
       </c>
     </row>
-    <row r="358" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="358" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A358" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B358">
         <v>4</v>
@@ -9147,9 +9147,9 @@
         <v>-4.0507937659991704</v>
       </c>
     </row>
-    <row r="359" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="359" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A359" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B359">
         <v>9147</v>
@@ -9167,9 +9167,9 @@
         <v>-5.5657775371856104</v>
       </c>
     </row>
-    <row r="360" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="360" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A360" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B360">
         <v>1154</v>
@@ -9187,9 +9187,9 @@
         <v>-5.9885658281460596</v>
       </c>
     </row>
-    <row r="361" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="361" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A361" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="B361">
         <v>1</v>
@@ -9207,9 +9207,9 @@
         <v>-4.9980899100669598</v>
       </c>
     </row>
-    <row r="362" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="362" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A362" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B362">
         <v>5</v>
@@ -9227,9 +9227,9 @@
         <v>-4.0507937659991704</v>
       </c>
     </row>
-    <row r="363" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="363" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A363" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B363">
         <v>2171</v>
@@ -9247,9 +9247,9 @@
         <v>-5.9885658281460596</v>
       </c>
     </row>
-    <row r="364" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="364" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A364" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B364">
         <v>1</v>
@@ -9267,9 +9267,9 @@
         <v>-4.32007128012346</v>
       </c>
     </row>
-    <row r="365" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="365" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A365" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B365">
         <v>15</v>
@@ -9287,9 +9287,9 @@
         <v>-5.3964670852082</v>
       </c>
     </row>
-    <row r="366" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="366" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A366" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B366">
         <v>48</v>
@@ -9307,9 +9307,9 @@
         <v>-5.7336160541347603</v>
       </c>
     </row>
-    <row r="367" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="367" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A367" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B367">
         <v>1</v>

</xml_diff>